<commit_message>
CI: mod job is required now that it passed on a runner; record G2-06/07 done
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G6" s="50" t="inlineStr">
         <is>
-          <t>tests/ (npm test, 19 pass); plugins/session-agents (claude plugin test, 15 pass); docs/PROGRESS.md</t>
+          <t>https://github.com/d10or/workspace-guardian (CI run 39390316230 green); tests/; docs/PROGRESS.md</t>
         </is>
       </c>
       <c r="H6" s="50" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H24" s="18" t="inlineStr">
@@ -3144,8 +3144,16 @@
           <t>.github/workflows/ci.yml passes on both OSes</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr"/>
-      <c r="J24" s="18" t="inlineStr"/>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>https://github.com/d10or/workspace-guardian/actions/runs/39390316230</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>3 jobs green on first push</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
@@ -3180,7 +3188,7 @@
       </c>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
@@ -3188,10 +3196,14 @@
           <t>LICENSE file; package.json license updated</t>
         </is>
       </c>
-      <c r="I25" s="18" t="inlineStr"/>
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>LICENSE; package.json</t>
+        </is>
+      </c>
       <c r="J25" s="18" t="inlineStr">
         <is>
-          <t>free core must stay open for awesome-claude-code</t>
+          <t>MIT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close G2, prepare G3–G6: safety audit, demo script, alpha guide, release docs, pricing, mod 0.15.0
- docs/SAFETY_AUDIT.md: P0 criteria mapped to code and tests
- demo/scenarios.sh + docs/DEMO.md: clean / risky / handoff scenarios
- docs/ALPHA_GUIDE.md, docs/ALPHA_OUTREACH.md (G3)
- CHANGELOG.md, docs/PRIVACY.md, docs/RELEASE_CHECKLIST.md, issue templates (G4)
- docs/PRICING.md: free/Pro boundary, two price messages, checkout plan (G5)
- docs/DECISION_MEMO.md template (G6)
- mod 0.15.0: per-session message files, timer guard; CI checks version match
- tracker, progress log and plan record gate statuses

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -1756,17 +1756,17 @@
       </c>
       <c r="F6" s="50" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G6" s="50" t="inlineStr">
         <is>
-          <t>https://github.com/d10or/workspace-guardian (CI run 39390316230 green); tests/; docs/PROGRESS.md</t>
+          <t>docs/SAFETY_AUDIT.md; tests/ (19 CLI + 16 mod + hook); CI green; demo/scenarios.sh; tag v0.1.0</t>
         </is>
       </c>
       <c r="H6" s="50" t="inlineStr">
         <is>
-          <t>Started early (2026-10-20) from the existing session-agents mod. CLI inspect/task/check/handoff done; mod v0.14.1 with task ownership done. Owed: CI green on macOS+Linux, license, demo recording.</t>
+          <t>Closed 2026-10-20, ahead of the Oct 26–Nov 1 window. All five deliverables with evidence. Demo recordings (G2-09) prepared via demo/scenarios.sh; the clips themselves are the founder's.</t>
         </is>
       </c>
     </row>
@@ -1798,11 +1798,19 @@
       </c>
       <c r="F7" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G7" s="50" t="str"/>
-      <c r="H7" s="50" t="str"/>
+          <t>Ready — awaiting testers</t>
+        </is>
+      </c>
+      <c r="G7" s="50" t="inlineStr">
+        <is>
+          <t>docs/ALPHA_GUIDE.md; docs/ALPHA_OUTREACH.md</t>
+        </is>
+      </c>
+      <c r="H7" s="50" t="inlineStr">
+        <is>
+          <t>Everything a tester needs exists. Exit needs 5 real testers observed; cannot be closed without them.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="56" customHeight="1">
       <c r="A8" s="50" t="inlineStr">
@@ -1832,11 +1840,19 @@
       </c>
       <c r="F8" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G8" s="50" t="str"/>
-      <c r="H8" s="50" t="str"/>
+          <t>Ready — awaiting launch</t>
+        </is>
+      </c>
+      <c r="G8" s="50" t="inlineStr">
+        <is>
+          <t>CHANGELOG.md; docs/PRIVACY.md; docs/RELEASE_CHECKLIST.md; .github/ISSUE_TEMPLATE; release v0.1.0</t>
+        </is>
+      </c>
+      <c r="H8" s="50" t="inlineStr">
+        <is>
+          <t>Public repo, tagged release, docs, privacy, issue templates done. Exit needs the directory submission, demo clips posted, and ≥50 verified installs measured.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="56" customHeight="1">
       <c r="A9" s="50" t="inlineStr">
@@ -1866,11 +1882,19 @@
       </c>
       <c r="F9" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G9" s="50" t="str"/>
-      <c r="H9" s="50" t="str"/>
+          <t>Ready — awaiting build + checkout</t>
+        </is>
+      </c>
+      <c r="G9" s="50" t="inlineStr">
+        <is>
+          <t>docs/PRICING.md</t>
+        </is>
+      </c>
+      <c r="H9" s="50" t="inlineStr">
+        <is>
+          <t>Free/Pro boundary, two price messages, checkout/fulfilment/refund plan written. Exit needs Pro features behind a license, a live checkout, and real buyers.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="56" customHeight="1">
       <c r="A10" s="50" t="inlineStr">
@@ -1900,11 +1924,19 @@
       </c>
       <c r="F10" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G10" s="50" t="str"/>
-      <c r="H10" s="50" t="str"/>
+          <t>Template ready</t>
+        </is>
+      </c>
+      <c r="G10" s="50" t="inlineStr">
+        <is>
+          <t>docs/DECISION_MEMO.md</t>
+        </is>
+      </c>
+      <c r="H10" s="50" t="inlineStr">
+        <is>
+          <t>Memo template with thresholds and formulas. Exit is the dated decision on 2026-11-29 with frozen metrics.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="n"/>
@@ -2644,7 +2676,7 @@
       </c>
       <c r="G13" s="50" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H13" s="50" t="inlineStr">
@@ -2654,12 +2686,12 @@
       </c>
       <c r="I13" s="50" t="inlineStr">
         <is>
-          <t>tests/fixtures.test.ts; tests/cli.test.ts</t>
+          <t>docs/SAFETY_AUDIT.md; tests/</t>
         </is>
       </c>
       <c r="J13" s="50" t="inlineStr">
         <is>
-          <t>19 node tests + 15 mod tests; safety audit still owed</t>
+          <t>19 CLI + 16 mod + hook tests; audit row by row</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2728,7 @@
       </c>
       <c r="G14" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H14" s="50" t="inlineStr">
@@ -2704,8 +2736,12 @@
           <t>New user can run workflow from clean clone</t>
         </is>
       </c>
-      <c r="I14" s="50" t="str"/>
-      <c r="J14" s="50" t="str"/>
+      <c r="I14" s="50" t="inlineStr">
+        <is>
+          <t>docs/ALPHA_GUIDE.md</t>
+        </is>
+      </c>
+      <c r="J14" s="50" t="inlineStr"/>
     </row>
     <row r="15" ht="39" customHeight="1">
       <c r="A15" s="50" t="inlineStr">
@@ -2740,7 +2776,7 @@
       </c>
       <c r="G15" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="H15" s="50" t="inlineStr">
@@ -2748,8 +2784,16 @@
           <t>Five distinct qualified volunteers</t>
         </is>
       </c>
-      <c r="I15" s="50" t="str"/>
-      <c r="J15" s="50" t="str"/>
+      <c r="I15" s="50" t="inlineStr">
+        <is>
+          <t>docs/ALPHA_OUTREACH.md</t>
+        </is>
+      </c>
+      <c r="J15" s="50" t="inlineStr">
+        <is>
+          <t>targets + message drafted; sending is the founder's</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="39" customHeight="1">
       <c r="A16" s="50" t="inlineStr">
@@ -2828,7 +2872,7 @@
       </c>
       <c r="G17" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H17" s="50" t="inlineStr">
@@ -2836,8 +2880,12 @@
           <t>License, docs, privacy, changelog, smoke test</t>
         </is>
       </c>
-      <c r="I17" s="50" t="str"/>
-      <c r="J17" s="50" t="str"/>
+      <c r="I17" s="50" t="inlineStr">
+        <is>
+          <t>docs/RELEASE_CHECKLIST.md; release v0.1.0</t>
+        </is>
+      </c>
+      <c r="J17" s="50" t="inlineStr"/>
     </row>
     <row r="18" ht="39" customHeight="1">
       <c r="A18" s="50" t="inlineStr">
@@ -2872,7 +2920,7 @@
       </c>
       <c r="G18" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="H18" s="50" t="inlineStr">
@@ -2880,8 +2928,16 @@
           <t>Screens include overlap and handoff scenarios</t>
         </is>
       </c>
-      <c r="I18" s="50" t="str"/>
-      <c r="J18" s="50" t="str"/>
+      <c r="I18" s="50" t="inlineStr">
+        <is>
+          <t>docs/DEMO.md</t>
+        </is>
+      </c>
+      <c r="J18" s="50" t="inlineStr">
+        <is>
+          <t>script ready; recordings owed</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="39" customHeight="1">
       <c r="A19" s="50" t="inlineStr">
@@ -2916,7 +2972,7 @@
       </c>
       <c r="G19" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="H19" s="50" t="inlineStr">
@@ -2924,8 +2980,16 @@
           <t>Channels logged; follows community rules</t>
         </is>
       </c>
-      <c r="I19" s="50" t="str"/>
-      <c r="J19" s="50" t="str"/>
+      <c r="I19" s="50" t="inlineStr">
+        <is>
+          <t>docs/RESEARCH_G1.md §4 channel list</t>
+        </is>
+      </c>
+      <c r="J19" s="50" t="inlineStr">
+        <is>
+          <t>directory submission + Reddit/HN/X posts are the founder's</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="39" customHeight="1">
       <c r="A20" s="50" t="inlineStr">
@@ -2960,7 +3024,7 @@
       </c>
       <c r="G20" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="H20" s="50" t="inlineStr">
@@ -2968,8 +3032,16 @@
           <t>Distinct Pro benefit; non-leading buyer feedback</t>
         </is>
       </c>
-      <c r="I20" s="50" t="str"/>
-      <c r="J20" s="50" t="str"/>
+      <c r="I20" s="50" t="inlineStr">
+        <is>
+          <t>docs/PRICING.md</t>
+        </is>
+      </c>
+      <c r="J20" s="50" t="inlineStr">
+        <is>
+          <t>boundary + 2 price messages written; Pro build + checkout owed</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="39" customHeight="1">
       <c r="A21" s="50" t="inlineStr">
@@ -3092,7 +3164,7 @@
       </c>
       <c r="G23" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Template</t>
         </is>
       </c>
       <c r="H23" s="50" t="inlineStr">
@@ -3100,8 +3172,12 @@
           <t>Decision, reasons, 30-day next actions</t>
         </is>
       </c>
-      <c r="I23" s="50" t="str"/>
-      <c r="J23" s="50" t="str"/>
+      <c r="I23" s="50" t="inlineStr">
+        <is>
+          <t>docs/DECISION_MEMO.md</t>
+        </is>
+      </c>
+      <c r="J23" s="50" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
@@ -3240,7 +3316,7 @@
       </c>
       <c r="G26" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H26" s="18" t="inlineStr">
@@ -3248,10 +3324,14 @@
           <t>claude plugin test green</t>
         </is>
       </c>
-      <c r="I26" s="18" t="inlineStr"/>
+      <c r="I26" s="18" t="inlineStr">
+        <is>
+          <t>plugins/session-agents v0.15.0; .github/workflows/ci.yml</t>
+        </is>
+      </c>
       <c r="J26" s="18" t="inlineStr">
         <is>
-          <t>MOD_REVIEW findings 11 remainder</t>
+          <t>messages per session, timer guard, version check in CI</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3368,7 @@
       </c>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="H27" s="18" t="inlineStr">
@@ -3296,8 +3376,16 @@
           <t>2 short recordings</t>
         </is>
       </c>
-      <c r="I27" s="18" t="inlineStr"/>
-      <c r="J27" s="18" t="inlineStr"/>
+      <c r="I27" s="18" t="inlineStr">
+        <is>
+          <t>demo/scenarios.sh; docs/DEMO.md</t>
+        </is>
+      </c>
+      <c r="J27" s="18" t="inlineStr">
+        <is>
+          <t>script builds all 3 scenarios; founder records the clips</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="18" t="n"/>
@@ -6080,13 +6168,41 @@
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="50" t="n"/>
-      <c r="B9" s="50" t="n"/>
-      <c r="C9" s="50" t="n"/>
-      <c r="D9" s="50" t="n"/>
-      <c r="E9" s="50" t="n"/>
-      <c r="F9" s="50" t="n"/>
-      <c r="G9" s="50" t="n"/>
+      <c r="A9" s="50" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C9" s="50" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="D9" s="50" t="inlineStr">
+        <is>
+          <t>G2 closed with evidence; G3–G6 artifacts prepared; G3–G6 exits stay open until real testers, installs and buyers exist</t>
+        </is>
+      </c>
+      <c r="E9" s="50" t="inlineStr">
+        <is>
+          <t>docs/SAFETY_AUDIT.md, CI, release v0.1.0; MASTER_PLAN §5 pass criteria need external evidence that cannot be produced internally</t>
+        </is>
+      </c>
+      <c r="F9" s="50" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="G9" s="50" t="inlineStr">
+        <is>
+          <t>Send alpha outreach (G3-02); record demo clips (G2-09)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="50" t="n"/>

</xml_diff>

<commit_message>
README: embed the three approved demo recordings; record G2-09 terminal clips done
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -2920,7 +2920,7 @@
       </c>
       <c r="G18" s="50" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done (terminal clips)</t>
         </is>
       </c>
       <c r="H18" s="50" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="I18" s="50" t="inlineStr">
         <is>
-          <t>docs/DEMO.md</t>
+          <t>demo/recordings/</t>
         </is>
       </c>
       <c r="J18" s="50" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done (terminal clips)</t>
         </is>
       </c>
       <c r="H27" s="18" t="inlineStr">
@@ -3378,12 +3378,12 @@
       </c>
       <c r="I27" s="18" t="inlineStr">
         <is>
-          <t>demo/scenarios.sh; docs/DEMO.md</t>
+          <t>demo/recordings/*.gif; README "See it"</t>
         </is>
       </c>
       <c r="J27" s="18" t="inlineStr">
         <is>
-          <t>script builds all 3 scenarios; founder records the clips</t>
+          <t>3 terminal clips recorded by Claude, approved by founder 2026-10-20; the in-Claude-Code Allow/Deny clip is still the founder's</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Relicense: MIT → PolyForm Shield 1.0.0 (source-available, noncompete); paid features move to a private repo
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -5689,7 +5689,7 @@
       </c>
       <c r="H11" s="50" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Mitigated: PolyForm Shield on public repo; Pro private; provenance notes record the MIT window (0 clones)</t>
         </is>
       </c>
     </row>
@@ -6205,13 +6205,41 @@
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="50" t="n"/>
-      <c r="B10" s="50" t="n"/>
-      <c r="C10" s="50" t="n"/>
-      <c r="D10" s="50" t="n"/>
-      <c r="E10" s="50" t="n"/>
-      <c r="F10" s="50" t="n"/>
-      <c r="G10" s="50" t="n"/>
+      <c r="A10" s="50" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B10" s="50" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C10" s="50" t="inlineStr">
+        <is>
+          <t>G4/G5</t>
+        </is>
+      </c>
+      <c r="D10" s="50" t="inlineStr">
+        <is>
+          <t>Relicense public repo MIT → PolyForm Shield 1.0.0; paid features in private repo workspace-guardian-pro; drop awesome-claude-code channel</t>
+        </is>
+      </c>
+      <c r="E10" s="50" t="inlineStr">
+        <is>
+          <t>Founder requirement: nobody may clone the project and offer it as their own. GitHub traffic at change: 0 clones, 0 forks, 0 stars. Shield allows use at work, forbids competing products.</t>
+        </is>
+      </c>
+      <c r="F10" s="50" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="G10" s="50" t="inlineStr">
+        <is>
+          <t>Create pro repo skeleton + license-key design (done 2026-10-20)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="50" t="n"/>

</xml_diff>

<commit_message>
CLI 0.2.0: offline Pro license (guardian license), Pro loader in check, policy/hotspot files from the main worktree
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -3024,7 +3024,7 @@
       </c>
       <c r="G20" s="50" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H20" s="50" t="inlineStr">
@@ -3034,12 +3034,12 @@
       </c>
       <c r="I20" s="50" t="inlineStr">
         <is>
-          <t>docs/PRICING.md</t>
+          <t>workspace-guardian-pro@400c0cb; src/lib/license.ts; tests/pro.test.ts</t>
         </is>
       </c>
       <c r="J20" s="50" t="inlineStr">
         <is>
-          <t>boundary + 2 price messages written; Pro build + checkout owed</t>
+          <t>Pro 0.1.0 built + verified with a signed key 2026-10-23; checkout page and price messages still owed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
guardian pro install|status|remove; Lemon Squeezy checkout guide; decision D7
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -3076,7 +3076,7 @@
       </c>
       <c r="G21" s="50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready — founder setup</t>
         </is>
       </c>
       <c r="H21" s="50" t="inlineStr">
@@ -3084,8 +3084,16 @@
           <t>Successful test order, delivery and policy</t>
         </is>
       </c>
-      <c r="I21" s="50" t="str"/>
-      <c r="J21" s="50" t="str"/>
+      <c r="I21" s="50" t="inlineStr">
+        <is>
+          <t>docs/CHECKOUT_LEMONSQUEEZY.md; workspace-guardian-pro scripts/pack.sh, scripts/fulfil.ts</t>
+        </is>
+      </c>
+      <c r="J21" s="50" t="inlineStr">
+        <is>
+          <t>engineering done 2026-10-23; store creation, test purchase and refund are the founder's</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="39" customHeight="1">
       <c r="A22" s="50" t="inlineStr">
@@ -6242,13 +6250,41 @@
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="50" t="n"/>
-      <c r="B11" s="50" t="n"/>
-      <c r="C11" s="50" t="n"/>
-      <c r="D11" s="50" t="n"/>
-      <c r="E11" s="50" t="n"/>
-      <c r="F11" s="50" t="n"/>
-      <c r="G11" s="50" t="n"/>
+      <c r="A11" s="50" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C11" s="50" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="D11" s="50" t="inlineStr">
+        <is>
+          <t>Checkout provider: Lemon Squeezy; manual key fulfilment during pilot; webhook signer deferred</t>
+        </is>
+      </c>
+      <c r="E11" s="50" t="inlineStr">
+        <is>
+          <t>Merchant of record (tax), file delivery, two price variants on one product; 3-buyer pass mark makes manual fulfilment fine</t>
+        </is>
+      </c>
+      <c r="F11" s="50" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="G11" s="50" t="inlineStr">
+        <is>
+          <t>Set up store per docs/CHECKOUT_LEMONSQUEEZY.md; test purchase + refund</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="50" t="n"/>

</xml_diff>

<commit_message>
Founding price: Pro $1/month for 30 days or 100 buyers; store variant F, page copy, launch lines; decision D8
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -6287,13 +6287,41 @@
       </c>
     </row>
     <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="50" t="n"/>
-      <c r="B12" s="50" t="n"/>
-      <c r="C12" s="50" t="n"/>
-      <c r="D12" s="50" t="n"/>
-      <c r="E12" s="50" t="n"/>
-      <c r="F12" s="50" t="n"/>
-      <c r="G12" s="50" t="n"/>
+      <c r="A12" s="50" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B12" s="50" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C12" s="50" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="inlineStr">
+        <is>
+          <t>Founding price: Pro $1/month for first 30 days or 100 buyers, grandfathered; free core stays free and public</t>
+        </is>
+      </c>
+      <c r="E12" s="50" t="inlineStr">
+        <is>
+          <t>Paid users are the feedback cohort; no marketplace can sell a Claude Code mod; directory lists free plugins only; Lemon Squeezy nets ~$0.45/$1</t>
+        </is>
+      </c>
+      <c r="F12" s="50" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="G12" s="50" t="inlineStr">
+        <is>
+          <t>Create store with variant F; launch posts carry the founding line</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="50" t="n"/>

</xml_diff>

<commit_message>
Decision D9: Lemon Squeezy only; free Agensi skill wrapper deferred to after launch (G4-04)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -3396,16 +3396,52 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="n"/>
-      <c r="B28" s="18" t="n"/>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="18" t="n"/>
-      <c r="I28" s="18" t="n"/>
-      <c r="J28" s="18" t="n"/>
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>G4-04</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>Free SKILL.md wrapper for the CLI listed on Agensi.io (discovery for Cursor/Codex users)</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Engineering / founder</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="inlineStr">
+        <is>
+          <t>skill lists, points at repo + store; zero Pro content</t>
+        </is>
+      </c>
+      <c r="I28" s="18" t="inlineStr"/>
+      <c r="J28" s="18" t="inlineStr">
+        <is>
+          <t>after launch data exists; never Pro</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="18" t="n"/>
@@ -6324,13 +6360,41 @@
       </c>
     </row>
     <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="50" t="n"/>
-      <c r="B13" s="50" t="n"/>
-      <c r="C13" s="50" t="n"/>
-      <c r="D13" s="50" t="n"/>
-      <c r="E13" s="50" t="n"/>
-      <c r="F13" s="50" t="n"/>
-      <c r="G13" s="50" t="n"/>
+      <c r="A13" s="50" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="inlineStr">
+        <is>
+          <t>G4/G5</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>Sell only via Lemon Squeezy; list a free SKILL.md wrapper on Agensi.io after launch (discovery for Cursor/Codex users), never Pro</t>
+        </is>
+      </c>
+      <c r="E13" s="50" t="inlineStr">
+        <is>
+          <t>Agensi sells SKILL.md files only, via its own MCP connector, 30% fee; numbers self-reported; our Pro is a package + key</t>
+        </is>
+      </c>
+      <c r="F13" s="50" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="G13" s="50" t="inlineStr">
+        <is>
+          <t>Add backlog G4-04 after launch</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="50" t="n"/>

</xml_diff>

<commit_message>
checkpoint: hand-off point — founder runbook, continuity-kit backlog item, where we stopped
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -3444,16 +3444,52 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="n"/>
-      <c r="B29" s="18" t="n"/>
-      <c r="C29" s="18" t="n"/>
-      <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
-      <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="18" t="n"/>
-      <c r="I29" s="18" t="n"/>
-      <c r="J29" s="18" t="n"/>
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>G4-05</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>"Project Continuity Kit" skill pack (checkpoint/resume/gate + SessionStart hook + templates) sold on Agensi.io; later a "Shared checkout safety" skill</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>Engineering / founder</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H29" s="18" t="inlineStr">
+        <is>
+          <t>listed, priced $9–$19, zero Pro content, points at repo + store</t>
+        </is>
+      </c>
+      <c r="I29" s="18" t="inlineStr"/>
+      <c r="J29" s="18" t="inlineStr">
+        <is>
+          <t>side line + discovery; after launch posts</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="18" t="n"/>

</xml_diff>

<commit_message>
Research round 2: broader pain points, six-week market scan, 12-item roadmap; backlog R1–R10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_TRACKER.xlsx
+++ b/docs/EXECUTION_TRACKER.xlsx
@@ -3492,124 +3492,508 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="n"/>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="18" t="n"/>
-      <c r="I30" s="18" t="n"/>
-      <c r="J30" s="18" t="n"/>
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>Destructive-git guard: hold reset/checkout --/clean/stash/force-push when tree dirty or other sessions own paths; safety ref before allowed ops; guardian undo</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G30" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>tests: compound commands, dirty tree, other-session claim, safety ref restorable</t>
+        </is>
+      </c>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>docs/RESEARCH_G2_IMPROVEMENTS.md R1</t>
+        </is>
+      </c>
+      <c r="J30" s="18" t="inlineStr">
+        <is>
+          <t>pain #2</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="n"/>
-      <c r="B31" s="18" t="n"/>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="18" t="n"/>
-      <c r="I31" s="18" t="n"/>
-      <c r="J31" s="18" t="n"/>
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>Hold dialog v2: names owner @session, task, age; Ask owner / Proceed once / Stop</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="G31" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H31" s="18" t="inlineStr">
+        <is>
+          <t>kit test + live check</t>
+        </is>
+      </c>
+      <c r="I31" s="18" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="J31" s="18" t="inlineStr">
+        <is>
+          <t>opening 1</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="n"/>
-      <c r="B32" s="18" t="n"/>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="18" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>STALE evidence: handoff/plan mark stale when owned paths changed after fingerprint; refuse unverified done once per task</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="G32" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H32" s="18" t="inlineStr">
+        <is>
+          <t>fixture: edit after test run → STALE</t>
+        </is>
+      </c>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J32" s="18" t="inlineStr">
+        <is>
+          <t>pain #7</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="n"/>
-      <c r="B33" s="18" t="n"/>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="18" t="n"/>
-      <c r="J33" s="18" t="n"/>
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>Migrate shared limits/claims to $.store; sessions from claude agents --json; Jump via $.ui.view</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F33" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="G33" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H33" s="18" t="inlineStr">
+        <is>
+          <t>no JSON race files remain; tests green</t>
+        </is>
+      </c>
+      <c r="I33" s="18" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="J33" s="18" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
-      <c r="B34" s="18" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="18" t="n"/>
-      <c r="F34" s="18" t="n"/>
-      <c r="G34" s="18" t="n"/>
-      <c r="H34" s="18" t="n"/>
-      <c r="I34" s="18" t="n"/>
-      <c r="J34" s="18" t="n"/>
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>Preflight v2: merge-tree between worktree branches incl. working trees; "would conflict once X lands"; scored term in Pro plan</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="G34" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H34" s="18" t="inlineStr">
+        <is>
+          <t>fixtures with cross-branch conflicts</t>
+        </is>
+      </c>
+      <c r="I34" s="18" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="J34" s="18" t="inlineStr">
+        <is>
+          <t>opening 4</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="n"/>
-      <c r="B35" s="18" t="n"/>
-      <c r="C35" s="18" t="n"/>
-      <c r="D35" s="18" t="n"/>
-      <c r="E35" s="18" t="n"/>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18" t="n"/>
-      <c r="H35" s="18" t="n"/>
-      <c r="I35" s="18" t="n"/>
-      <c r="J35" s="18" t="n"/>
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D35" s="18" t="inlineStr">
+        <is>
+          <t>Compaction-safe task state: PreCompact snapshot, SessionStart re-inject, compacted-N-min badge</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="G35" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H35" s="18" t="inlineStr">
+        <is>
+          <t>state survives a forced compact</t>
+        </is>
+      </c>
+      <c r="I35" s="18" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="J35" s="18" t="inlineStr">
+        <is>
+          <t>pain #3</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="n"/>
-      <c r="B36" s="18" t="n"/>
-      <c r="C36" s="18" t="n"/>
-      <c r="D36" s="18" t="n"/>
-      <c r="E36" s="18" t="n"/>
-      <c r="F36" s="18" t="n"/>
-      <c r="G36" s="18" t="n"/>
-      <c r="H36" s="18" t="n"/>
-      <c r="I36" s="18" t="n"/>
-      <c r="J36" s="18" t="n"/>
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D36" s="18" t="inlineStr">
+        <is>
+          <t>Per-session usage attribution of the 5h window in the band</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="G36" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H36" s="18" t="inlineStr"/>
+      <c r="I36" s="18" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="J36" s="18" t="inlineStr">
+        <is>
+          <t>pain #1</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="n"/>
-      <c r="B37" s="18" t="n"/>
-      <c r="C37" s="18" t="n"/>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="18" t="n"/>
-      <c r="H37" s="18" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="B37" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C37" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>Permission ledger per session in the pane</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F37" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="G37" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H37" s="18" t="inlineStr"/>
+      <c r="I37" s="18" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="J37" s="18" t="inlineStr">
+        <is>
+          <t>pain #5</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="n"/>
-      <c r="B38" s="18" t="n"/>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18" t="n"/>
-      <c r="G38" s="18" t="n"/>
-      <c r="H38" s="18" t="n"/>
-      <c r="I38" s="18" t="n"/>
-      <c r="J38" s="18" t="n"/>
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>Secret guard on tool output + staged diffs</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F38" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="G38" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H38" s="18" t="inlineStr"/>
+      <c r="I38" s="18" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="J38" s="18" t="inlineStr">
+        <is>
+          <t>pain #10</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
-      <c r="B39" s="18" t="n"/>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-      <c r="G39" s="18" t="n"/>
-      <c r="H39" s="18" t="n"/>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B39" s="18" t="inlineStr">
+        <is>
+          <t>post-launch</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>Worktree lifecycle in inspect: age, owner, stale, base drift</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F39" s="18" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="G39" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H39" s="18" t="inlineStr"/>
+      <c r="I39" s="18" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="J39" s="18" t="inlineStr">
+        <is>
+          <t>pain #9</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="18" t="n"/>

</xml_diff>